<commit_message>
version 34 - Design and Implement Database migration, Implement Login and Register component
</commit_message>
<xml_diff>
--- a/Database_Architecture/Database_design_architecture.xlsx
+++ b/Database_Architecture/Database_design_architecture.xlsx
@@ -4,13 +4,24 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8280" activeTab="3"/>
+    <workbookView windowWidth="23040" windowHeight="9000" tabRatio="777" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
-    <sheet name="Structure" sheetId="2" r:id="rId2"/>
-    <sheet name="Relationship" sheetId="3" r:id="rId3"/>
-    <sheet name="Table" sheetId="4" r:id="rId4"/>
+    <sheet name="Relationship" sheetId="3" r:id="rId2"/>
+    <sheet name="Table_Interface_summarize" sheetId="5" r:id="rId3"/>
+    <sheet name="customers" sheetId="6" r:id="rId4"/>
+    <sheet name="phone" sheetId="7" r:id="rId5"/>
+    <sheet name="orders" sheetId="8" r:id="rId6"/>
+    <sheet name="order_details" sheetId="9" r:id="rId7"/>
+    <sheet name="inventory" sheetId="10" r:id="rId8"/>
+    <sheet name="coupons" sheetId="11" r:id="rId9"/>
+    <sheet name="payments" sheetId="12" r:id="rId10"/>
+    <sheet name="ware_houses" sheetId="13" r:id="rId11"/>
+    <sheet name="order_details_inventory" sheetId="14" r:id="rId12"/>
+    <sheet name="customer_coupons" sheetId="15" r:id="rId13"/>
+    <sheet name="order_coupons" sheetId="16" r:id="rId14"/>
+    <sheet name="NoSQLDatabase" sheetId="17" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="209">
   <si>
     <t>Model for SQL and No SQL combination</t>
   </si>
@@ -459,49 +470,269 @@
     <t>SQL and NO SQL relationship</t>
   </si>
   <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `customers` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `customer_id` INT AUTO_INCREMENT PRIMARY KEY,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `name` VARCHAR(100) NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `email` VARCHAR(100) NOT NULL UNIQUE,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `phone` VARCHAR(20),</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `address` VARCHAR(255),</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `created_at` DATETIME DEFAULT CURRENT_TIMESTAMP</t>
-  </si>
-  <si>
-    <t>) ENGINE=InnoDB DEFAULT CHARSET=utf8mb4;</t>
-  </si>
-  <si>
-    <t>Order</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `orders` (</t>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Operation</t>
+  </si>
+  <si>
+    <t>SQL function (Ex1)</t>
+  </si>
+  <si>
+    <t>Meaning Ex1</t>
+  </si>
+  <si>
+    <t>SQL function (Ex2)</t>
+  </si>
+  <si>
+    <t>Meaning Ex2</t>
+  </si>
+  <si>
+    <t>customers</t>
+  </si>
+  <si>
+    <t>Read</t>
+  </si>
+  <si>
+    <t>SELECT customer_id, username, email, address
+FROM customers
+WHERE customer_id = 3;</t>
+  </si>
+  <si>
+    <t>Get customer information (4 feature) with customer id is 3</t>
+  </si>
+  <si>
+    <t>SELECT customer_id, name, email
+FROM customers
+WHERE address = 'HCM City';</t>
+  </si>
+  <si>
+    <t>Get customer information (3 feature) with address is "HCM City"</t>
+  </si>
+  <si>
+    <t>Update</t>
+  </si>
+  <si>
+    <t>UPDATE customers
+SET email = 'bob.new@gmail.com',
+    address = 'Ho Chi Minh City'
+WHERE customer_id = 2;</t>
+  </si>
+  <si>
+    <t>SELECT c.customer_id, c.name, c.email, p.phone
+FROM customers c
+JOIN phone p ON c.customer_id = p.customer_id;</t>
+  </si>
+  <si>
+    <t>Get customer information with phone number (Join 2 table)</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t>INSERT INTO customers (customer_id, username, password, first_name, last_name, name, email, address, created_at)
+VALUES
+(6, 'alice01',  'hashed_pw_1', 'Alice',  'Nguyen',  'Alice Nguyen',  'alice@gmail.com', 'Hanoi',      '2024-01-05 10:15:00'),
+(10, 'eric_5',   'hashed_pw_5', 'Eric',   'Hoang',   'Eric Hoang',    'eric@outlook.com','Hue',        '2024-01-17 16:30:00');</t>
+  </si>
+  <si>
+    <t>Delete</t>
+  </si>
+  <si>
+    <t>DELETE FROM customers
+WHERE customer_id = 2;</t>
+  </si>
+  <si>
+    <t>Due to "ON DELETE CASCADE", so if customer id 2 is deleted, all phone number will be clear automatically</t>
+  </si>
+  <si>
+    <t>DELETE FROM customers
+WHERE address = 'Hanoi';</t>
+  </si>
+  <si>
+    <t>Delete all customer have address "Hanoi", Phone number will be deleted automatically due to config</t>
+  </si>
+  <si>
+    <t>SELECT phone
+FROM phone
+WHERE customer_id = 1;</t>
+  </si>
+  <si>
+    <t>Get all phone number of customer id 1</t>
+  </si>
+  <si>
+    <t>UPDATE phone
+SET phone = '0911002200'
+WHERE customer_id = 6 AND phone = '0901234567';</t>
+  </si>
+  <si>
+    <t>Change one phone number of 2 number of customer 6</t>
+  </si>
+  <si>
+    <t>INSERT INTO phone (customer_id, phone)
+VALUES
+(6, '0901234567'),
+(6, '0912345678'),
+(10, '0967778888');</t>
+  </si>
+  <si>
+    <t>INSERT INTO Phone (customer_id, phone)
+VALUES (2, '0909998888');</t>
+  </si>
+  <si>
+    <t>Add additional phone number for customer id 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DELETE FROM phone
+WHERE customer_id = 3 AND phone = '0931112222';
+</t>
+  </si>
+  <si>
+    <t>Delete 1 of 2 phone number of customer id 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DELETE FROM phone
+WHERE customer_id = 4;
+</t>
+  </si>
+  <si>
+    <t>Delete all phone number of customer id 4</t>
+  </si>
+  <si>
+    <t>orders</t>
+  </si>
+  <si>
+    <t>SELECT *
+FROM `orders`
+WHERE customer_id = 2;</t>
+  </si>
+  <si>
+    <t>Get order information of customer id 2</t>
+  </si>
+  <si>
+    <t>SELECT o.order_id, o.order_date, o.total_amount, o.status,
+       c.name, c.email
+FROM `orders` o
+JOIN customers c ON o.customer_id = c.customer_id;</t>
+  </si>
+  <si>
+    <t>Get order with customer information (join 2 table)</t>
+  </si>
+  <si>
+    <t>UPDATE `orders`
+SET status = 'completed'
+WHERE order_id = 2;</t>
+  </si>
+  <si>
+    <t>Update status based on order id 2</t>
+  </si>
+  <si>
+    <t>UPDATE `orders`
+SET total_amount = 999000
+WHERE order_id = 3;</t>
+  </si>
+  <si>
+    <t>Update total amount based on order id 3</t>
+  </si>
+  <si>
+    <t>INSERT INTO `orders` (order_id, customer_id, order_date, total_amount, status)
+VALUES
+(6, 3, NOW(), 450000, 'pending');</t>
+  </si>
+  <si>
+    <t>Add 1 new order for customer id 3</t>
+  </si>
+  <si>
+    <t>DELETE FROM `orders`
+WHERE order_id = 5;</t>
+  </si>
+  <si>
+    <t>Delete order id 5</t>
+  </si>
+  <si>
+    <t>DELETE FROM `orders`
+WHERE customer_id = 4;</t>
+  </si>
+  <si>
+    <t>Delete all order of customer id 4</t>
+  </si>
+  <si>
+    <t>order_details</t>
+  </si>
+  <si>
+    <t>SELECT order_id, quantity, unit_price
+FROM order_details
+WHERE order_detail_id = 3; -- Ví dụ: Truy vấn chi tiết đơn hàng có ID = 3</t>
+  </si>
+  <si>
+    <t>get order detail based on order detail id 3</t>
+  </si>
+  <si>
+    <t>SELECT *
+FROM order_details
+WHERE order_id = 2;</t>
+  </si>
+  <si>
+    <t>get order detail based on order id 2 (use foreign key)</t>
+  </si>
+  <si>
+    <t>UPDATE order_details
+SET quantity = 5, subtotal = 5 * 25.99 
+WHERE order_detail_id = 4;</t>
+  </si>
+  <si>
+    <t>update quatity and subtotal based on order details id 4</t>
+  </si>
+  <si>
+    <t>INSERT INTO order_details (order_id, payment_id, variant_id, quantity, unit_price, subtotal) VALUES
+(6, 6, 106, 4, 12.50, 50.00);</t>
+  </si>
+  <si>
+    <t>add new order details</t>
+  </si>
+  <si>
+    <t>DELETE FROM order_details
+WHERE order_detail_id = 5;</t>
+  </si>
+  <si>
+    <t>Delete order detail 5</t>
+  </si>
+  <si>
+    <t>inventory</t>
+  </si>
+  <si>
+    <t>coupons</t>
+  </si>
+  <si>
+    <t>payments</t>
+  </si>
+  <si>
+    <t>ware_houses</t>
+  </si>
+  <si>
+    <t>order_details_inventory</t>
+  </si>
+  <si>
+    <t>customer_coupons</t>
+  </si>
+  <si>
+    <t>order_coupons</t>
+  </si>
+  <si>
+    <t>Home table</t>
   </si>
   <si>
     <t>→ Quan hệ:</t>
   </si>
   <si>
-    <t xml:space="preserve">  `order_id` INT AUTO_INCREMENT PRIMARY KEY,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `customer_id` INT NOT NULL,</t>
-  </si>
-  <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">1:N giữa </t>
     </r>
     <r>
@@ -517,10 +748,42 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  `order_date` DATETIME DEFAULT CURRENT_TIMESTAMP,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `total_amount` DECIMAL(12,2) NOT NULL,</t>
+    <r>
+      <t xml:space="preserve">N:N giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Customer → Coupons</t>
+    </r>
+  </si>
+  <si>
+    <t>--&gt; customer_coupons table</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">N:N giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Coupons → Order</t>
+    </r>
+  </si>
+  <si>
+    <t>--&gt; order_coupons table</t>
   </si>
   <si>
     <r>
@@ -535,35 +798,34 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Order ↔ Payment</t>
+      <t>Payment ↔ Order</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  `status` ENUM('pending','processing','shipped','completed','cancelled') DEFAULT 'pending',</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  -- payment_id removed to avoid circular FK; payments -&gt; orders (1:1) bằng UNIQUE on payments.order_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_orders_customer` FOREIGN KEY (`customer_id`) REFERENCES `customers` (`customer_id`) ON DELETE RESTRICT ON UPDATE CASCADE</t>
-  </si>
-  <si>
-    <t>)</t>
-  </si>
-  <si>
-    <t>Order_detail</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `order_details` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `order_detail_id` INT AUTO_INCREMENT PRIMARY KEY,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `order_id` INT NOT NULL,</t>
-  </si>
-  <si>
     <r>
+      <t xml:space="preserve">N:1 giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Order_detail → Order</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">1:N giữa </t>
     </r>
     <r>
@@ -579,13 +841,49 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  `product_sku` VARCHAR(100) NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `variant_id` VARCHAR(100),</t>
-  </si>
-  <si>
     <r>
+      <t xml:space="preserve">1:N giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Payment → Order_detail</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">N:N giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Inventory → Order_detail</t>
+    </r>
+  </si>
+  <si>
+    <t>--&gt; order_details_inventory table</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Tham chiếu mềm </t>
     </r>
     <r>
@@ -620,61 +918,14 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  `quantity` INT NOT NULL DEFAULT 1,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `unit_price` DECIMAL(12,2) NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `subtotal` DECIMAL(12,2) AS (`quantity` * `unit_price`) STORED,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_orderdetails_order` FOREIGN KEY (`order_id`) REFERENCES `orders` (`order_id`) ON DELETE CASCADE ON UPDATE CASCADE</t>
-  </si>
-  <si>
-    <t>Payment</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `payments` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `payment_id` INT AUTO_INCREMENT PRIMARY KEY,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `method` ENUM('cash','credit_card','paypal','bank_transfer') NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `transaction_id` VARCHAR(255),</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `amount` DECIMAL(12,2) NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `status` ENUM('pending','success','failed','refund') DEFAULT 'pending',</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `payment_date` DATETIME DEFAULT CURRENT_TIMESTAMP,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_payments_order` FOREIGN KEY (`order_id`) REFERENCES `orders` (`order_id`) ON DELETE CASCADE ON UPDATE CASCADE,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `uq_payments_order` UNIQUE (`order_id`)  -- đảm bảo 1:1 giữa order và payment</t>
-  </si>
-  <si>
-    <t>Inventory</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `inventory` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `inventory_id` INT AUTO_INCREMENT PRIMARY KEY,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `warehouse_id` INT NOT NULL,</t>
-  </si>
-  <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">1:N giữa </t>
     </r>
     <r>
@@ -690,10 +941,30 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  `variant_id` VARCHAR(100) DEFAULT NULL,</t>
-  </si>
-  <si>
     <r>
+      <t xml:space="preserve">N:N giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>order_details → Inventory</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Tham chiếu mềm </t>
     </r>
     <r>
@@ -728,124 +999,41 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">  `quantity` INT NOT NULL DEFAULT 0,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `updated_at` DATETIME DEFAULT CURRENT_TIMESTAMP ON UPDATE CURRENT_TIMESTAMP,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_inventory_warehouse` FOREIGN KEY (`warehouse_id`) REFERENCES `ware_houses` (`warehouse_id`) ON DELETE RESTRICT ON UPDATE CASCADE,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  INDEX `idx_inventory_sku` (`product_sku`),</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  INDEX `idx_inventory_variant` (`variant_id`)</t>
-  </si>
-  <si>
-    <t>Ware_house</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `ware_houses` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `warehouse_id` INT AUTO_INCREMENT PRIMARY KEY,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `location` VARCHAR(255),</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `capacity` INT,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `manager_name` VARCHAR(100)</t>
-  </si>
-  <si>
-    <t>Coupons</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `coupons` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `coupon_id` INT AUTO_INCREMENT PRIMARY KEY,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `code` VARCHAR(50) NOT NULL UNIQUE,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `discount_type` ENUM('percent','amount') NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `discount_value` DECIMAL(10,2) NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `min_order_value` DECIMAL(10,2) DEFAULT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `max_discount_value` DECIMAL(10,2) DEFAULT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `valid_from` DATETIME NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `valid_to` DATETIME NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `usage_limit` INT DEFAULT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `per_user_limit` INT DEFAULT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `status` ENUM('active','expired','disabled') DEFAULT 'active',</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `created_at` DATETIME DEFAULT CURRENT_TIMESTAMP,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `updated_at` DATETIME DEFAULT CURRENT_TIMESTAMP ON UPDATE CURRENT_TIMESTAMP</t>
-  </si>
-  <si>
-    <t>Customer_Coupons (n–n giữa Customer và Coupons)</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `customer_coupons` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `coupon_id` INT NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `times_used` INT DEFAULT 0,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `last_used_at` DATETIME DEFAULT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  PRIMARY KEY (`customer_id`, `coupon_id`),</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_cc_customer` FOREIGN KEY (`customer_id`) REFERENCES `customers` (`customer_id`) ON DELETE CASCADE ON UPDATE CASCADE,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_cc_coupon` FOREIGN KEY (`coupon_id`) REFERENCES `coupons` (`coupon_id`) ON DELETE CASCADE ON UPDATE CASCADE</t>
-  </si>
-  <si>
-    <t>Order_Coupons (n–n giữa Order và Coupons)</t>
-  </si>
-  <si>
-    <t>CREATE TABLE IF NOT EXISTS `order_coupons` (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  `discount_applied` DECIMAL(12,2) DEFAULT 0,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  PRIMARY KEY (`order_id`, `coupon_id`),</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_oc_order` FOREIGN KEY (`order_id`) REFERENCES `orders` (`order_id`) ON DELETE CASCADE ON UPDATE CASCADE,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONSTRAINT `fk_oc_coupon` FOREIGN KEY (`coupon_id`) REFERENCES `coupons` (`coupon_id`) ON DELETE CASCADE ON UPDATE CASCADE</t>
+    <r>
+      <t xml:space="preserve">N:N giữa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Order</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Coupons</t>
+    </r>
   </si>
   <si>
     <t>II. DOCUMENT SCHEMA (NoSQL – MongoDB)</t>
@@ -942,19 +1130,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -966,8 +1146,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -982,11 +1162,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1118,12 +1306,42 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1312,12 +1530,304 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="29">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1438,13 +1948,13 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1456,141 +1966,294 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="27" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1598,6 +2261,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" quotePrefix="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" quotePrefix="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1875,53 +2544,6 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>635</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>553085</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>48260</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="635" y="635"/>
-          <a:ext cx="17621250" cy="6448425"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2361,20 +2983,20 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>635</xdr:colOff>
-      <xdr:row>165</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>267335</xdr:colOff>
-      <xdr:row>193</xdr:row>
-      <xdr:rowOff>5715</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>495935</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>84455</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2391,8 +3013,987 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="635" y="31356300"/>
+          <a:off x="770255" y="635"/>
+          <a:ext cx="4152900" cy="2827020"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>153035</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5036820" y="635"/>
+          <a:ext cx="6812280" cy="1615440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>73660</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>568960</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>158115</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="843280" y="7620"/>
+          <a:ext cx="4762500" cy="4173855"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5715</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>23495</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>31115</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5652135" y="23495"/>
+          <a:ext cx="5471160" cy="1653540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>635</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>473075</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>23495</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="770255" y="635"/>
+          <a:ext cx="7787640" cy="4777740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>168910</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>10160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>138430</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>109220</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8863330" y="10160"/>
+          <a:ext cx="6065520" cy="1562100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>116840</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>178435</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="777240" y="7620"/>
+          <a:ext cx="9862820" cy="3828415"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>236220</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>259080</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>137795</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10759440" y="635"/>
+          <a:ext cx="4899660" cy="1600200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>78105</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>914400</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2750820" y="15554325"/>
           <a:ext cx="7581900" cy="5095875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>601980</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>225425</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>23495</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="601980" y="198120"/>
+          <a:ext cx="5879465" cy="3117215"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>635</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>198755</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="635" y="3413760"/>
+          <a:ext cx="13159740" cy="1668780"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>412115</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>18415</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="777240" y="7620"/>
+          <a:ext cx="5890895" cy="3119755"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>61595</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6896100" y="635"/>
+          <a:ext cx="3901440" cy="2438400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>281940</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="769620" y="0"/>
+          <a:ext cx="4549140" cy="2834640"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>594360</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>472440</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>137795</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5631180" y="635"/>
+          <a:ext cx="6583680" cy="1600200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>635</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>396875</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>183515</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="770255" y="635"/>
+          <a:ext cx="5882640" cy="2926080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>365760</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>53975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6880860" y="635"/>
+          <a:ext cx="7665720" cy="1699260"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>635</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>556895</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>69215</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="770255" y="635"/>
+          <a:ext cx="4213860" cy="4457700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>107315</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5013960" y="635"/>
+          <a:ext cx="8084820" cy="1569720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>53340</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>69215</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="822960" y="635"/>
+          <a:ext cx="6339840" cy="4640580"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>635</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>473075</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="770255" y="4373880"/>
+          <a:ext cx="14493240" cy="1485900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>635</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>175895</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>137795</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="770255" y="635"/>
+          <a:ext cx="8100060" cy="3611880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>635</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>610235</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="770255" y="3695700"/>
+          <a:ext cx="7924800" cy="1706880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2691,7 +4292,7 @@
       </c>
     </row>
     <row r="6" spans="4:4">
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="57" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2699,15 +4300,15 @@
       <c r="D7" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="58" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="4:6">
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="59" t="s">
         <v>7</v>
       </c>
       <c r="F8" t="s">
@@ -2715,8 +4316,8 @@
       </c>
     </row>
     <row r="9" spans="4:6">
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
       <c r="F9" t="s">
         <v>9</v>
       </c>
@@ -2755,7 +4356,7 @@
       </c>
     </row>
     <row r="17" spans="4:4">
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="57" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2763,7 +4364,7 @@
       <c r="D18" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="58" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2771,7 +4372,7 @@
       <c r="D19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="58" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2791,7 +4392,7 @@
       </c>
     </row>
     <row r="24" spans="4:4">
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="57" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2799,7 +4400,7 @@
       <c r="D25" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="58" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2807,7 +4408,7 @@
       <c r="D26" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="58" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2840,7 +4441,7 @@
       <c r="D33" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="58" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2848,7 +4449,7 @@
       <c r="D34" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="58" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2886,7 +4487,7 @@
       <c r="D42" t="s">
         <v>4</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="58" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2899,7 +4500,7 @@
       <c r="D44" t="s">
         <v>19</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="58" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2922,7 +4523,7 @@
       <c r="D49" t="s">
         <v>4</v>
       </c>
-      <c r="E49" s="7" t="s">
+      <c r="E49" s="58" t="s">
         <v>38</v>
       </c>
     </row>
@@ -3119,7 +4720,7 @@
       <c r="F66" t="s">
         <v>64</v>
       </c>
-      <c r="G66" s="9" t="s">
+      <c r="G66" s="60" t="s">
         <v>78</v>
       </c>
       <c r="H66" t="s">
@@ -3232,12 +4833,373 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4" spans="16:16">
+      <c r="P4" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" spans="16:16">
+      <c r="P6" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="16:16">
+      <c r="P7" s="7" t="s">
+        <v>176</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="9:9">
+      <c r="I11" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13" spans="9:9">
+      <c r="I13" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="7" tint="0.8"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="7" tint="0.8"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="7" tint="0.8"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="5" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" ht="25.8" spans="2:2">
+      <c r="B3" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="5" ht="21" spans="2:2">
+      <c r="B5" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" spans="3:3">
+      <c r="C7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="3:3">
+      <c r="C8" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="9" spans="3:3">
+      <c r="C9" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="10" spans="3:3">
+      <c r="C10" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="11" spans="3:3">
+      <c r="C11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="3:3">
+      <c r="C12" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="3:3">
+      <c r="C13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="3:3">
+      <c r="C14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="3:3">
+      <c r="C15" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="16" spans="3:3">
+      <c r="C16" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="19" ht="21" spans="2:2">
+      <c r="B19" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3">
+      <c r="C21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3">
+      <c r="C22" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3">
+      <c r="C23" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3">
+      <c r="C24" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3">
+      <c r="C25" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3">
+      <c r="C26" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="27" spans="3:3">
+      <c r="C27" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="28" spans="3:3">
+      <c r="C28" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3">
+      <c r="C29" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="31" ht="21" spans="2:2">
+      <c r="B31" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3">
+      <c r="C33" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3">
+      <c r="C34" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3">
+      <c r="C35" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="36" spans="3:3">
+      <c r="C36" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="37" spans="3:3">
+      <c r="C37" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="38" spans="3:3">
+      <c r="C38" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="39" spans="3:3">
+      <c r="C39" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="40" spans="3:3">
+      <c r="C40" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="41" spans="3:3">
+      <c r="C41" t="s">
+        <v>196</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
+  <dimension ref="A2:A61"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2" ht="25.8" spans="1:1">
+      <c r="A2" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" ht="25.8" spans="1:1">
+      <c r="A38" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="61" ht="25.8" spans="1:1">
+      <c r="A61" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>
@@ -3246,26 +5208,622 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A2:A61"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <sheetPr>
+    <tabColor theme="9" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:F45"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" width="25.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="10.7777777777778" customWidth="1"/>
+    <col min="3" max="3" width="100.777777777778" style="8" customWidth="1"/>
+    <col min="4" max="4" width="40.7777777777778" style="8" customWidth="1"/>
+    <col min="5" max="5" width="80.7777777777778" style="8" customWidth="1"/>
+    <col min="6" max="6" width="40.7777777777778" style="8" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" ht="25.8" spans="1:1">
-      <c r="A2" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="38" ht="25.8" spans="1:1">
-      <c r="A38" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="61" ht="25.8" spans="1:1">
-      <c r="A61" s="4" t="s">
-        <v>98</v>
-      </c>
+    <row r="1" ht="15.15" spans="1:6">
+      <c r="A1" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" ht="43.2" spans="1:6">
+      <c r="A2" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" ht="57.6" spans="1:6">
+      <c r="A3" s="21"/>
+      <c r="B3" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="24"/>
+      <c r="E3" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3" s="26" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" ht="57.6" spans="1:6">
+      <c r="A4" s="21"/>
+      <c r="B4" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="28"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="30"/>
+    </row>
+    <row r="5" ht="43.95" spans="1:6">
+      <c r="A5" s="31"/>
+      <c r="B5" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="F5" s="36" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" ht="43.2" spans="1:6">
+      <c r="A6" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="E6" s="38"/>
+      <c r="F6" s="39"/>
+    </row>
+    <row r="7" ht="43.2" spans="1:6">
+      <c r="A7" s="21"/>
+      <c r="B7" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="25"/>
+      <c r="F7" s="40"/>
+    </row>
+    <row r="8" ht="72" spans="1:6">
+      <c r="A8" s="21"/>
+      <c r="B8" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="24"/>
+      <c r="E8" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" ht="43.95" spans="1:6">
+      <c r="A9" s="31"/>
+      <c r="B9" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>129</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>130</v>
+      </c>
+      <c r="E9" s="43" t="s">
+        <v>131</v>
+      </c>
+      <c r="F9" s="44" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10" ht="57.6" spans="1:6">
+      <c r="A10" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" ht="43.2" spans="1:6">
+      <c r="A11" s="21"/>
+      <c r="B11" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="D11" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="F11" s="40" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" ht="43.2" spans="1:6">
+      <c r="A12" s="21"/>
+      <c r="B12" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="E12" s="46"/>
+      <c r="F12" s="40"/>
+    </row>
+    <row r="13" ht="29.55" spans="1:6">
+      <c r="A13" s="31"/>
+      <c r="B13" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="D13" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="F13" s="44" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14" ht="43.2" spans="1:6">
+      <c r="A14" s="47" t="s">
+        <v>148</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>150</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="15" ht="43.2" spans="1:6">
+      <c r="A15" s="48"/>
+      <c r="B15" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="E15" s="46"/>
+      <c r="F15" s="40"/>
+    </row>
+    <row r="16" ht="28.8" spans="1:6">
+      <c r="A16" s="48"/>
+      <c r="B16" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>156</v>
+      </c>
+      <c r="E16" s="46"/>
+      <c r="F16" s="40"/>
+    </row>
+    <row r="17" ht="29.55" spans="1:6">
+      <c r="A17" s="49"/>
+      <c r="B17" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="D17" s="42" t="s">
+        <v>158</v>
+      </c>
+      <c r="E17" s="50"/>
+      <c r="F17" s="44"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C18" s="51"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="39"/>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="21"/>
+      <c r="B19" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="52"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="40"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="21"/>
+      <c r="B20" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" s="52"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="40"/>
+    </row>
+    <row r="21" ht="15.15" spans="1:6">
+      <c r="A21" s="31"/>
+      <c r="B21" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" s="53"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="44"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" s="51"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="39"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="21"/>
+      <c r="B23" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C23" s="52"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="40"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="21"/>
+      <c r="B24" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C24" s="52"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="40"/>
+    </row>
+    <row r="25" ht="15.15" spans="1:6">
+      <c r="A25" s="31"/>
+      <c r="B25" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C25" s="53"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="44"/>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="51"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="39"/>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="21"/>
+      <c r="B27" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="52"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="40"/>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="21"/>
+      <c r="B28" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C28" s="52"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="40"/>
+    </row>
+    <row r="29" ht="15.15" spans="1:6">
+      <c r="A29" s="31"/>
+      <c r="B29" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C29" s="53"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="44"/>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C30" s="51"/>
+      <c r="D30" s="37"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="39"/>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="21"/>
+      <c r="B31" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C31" s="52"/>
+      <c r="D31" s="45"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="40"/>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="21"/>
+      <c r="B32" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C32" s="52"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="40"/>
+    </row>
+    <row r="33" ht="15.15" spans="1:6">
+      <c r="A33" s="31"/>
+      <c r="B33" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C33" s="53"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="44"/>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="54" t="s">
+        <v>163</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" s="51"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="39"/>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="55"/>
+      <c r="B35" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C35" s="52"/>
+      <c r="D35" s="45"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="40"/>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="55"/>
+      <c r="B36" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C36" s="52"/>
+      <c r="D36" s="45"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="40"/>
+    </row>
+    <row r="37" ht="15.15" spans="1:6">
+      <c r="A37" s="56"/>
+      <c r="B37" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C37" s="53"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="44"/>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="51"/>
+      <c r="D38" s="37"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="39"/>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="55"/>
+      <c r="B39" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C39" s="52"/>
+      <c r="D39" s="45"/>
+      <c r="E39" s="46"/>
+      <c r="F39" s="40"/>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="55"/>
+      <c r="B40" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C40" s="52"/>
+      <c r="D40" s="45"/>
+      <c r="E40" s="46"/>
+      <c r="F40" s="40"/>
+    </row>
+    <row r="41" ht="15.15" spans="1:6">
+      <c r="A41" s="56"/>
+      <c r="B41" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C41" s="53"/>
+      <c r="D41" s="42"/>
+      <c r="E41" s="50"/>
+      <c r="F41" s="44"/>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="54" t="s">
+        <v>165</v>
+      </c>
+      <c r="B42" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C42" s="51"/>
+      <c r="D42" s="37"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="39"/>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="55"/>
+      <c r="B43" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="52"/>
+      <c r="D43" s="45"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="40"/>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="55"/>
+      <c r="B44" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C44" s="52"/>
+      <c r="D44" s="45"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="40"/>
+    </row>
+    <row r="45" ht="15.15" spans="1:6">
+      <c r="A45" s="56"/>
+      <c r="B45" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C45" s="53"/>
+      <c r="D45" s="42"/>
+      <c r="E45" s="50"/>
+      <c r="F45" s="44"/>
     </row>
   </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A45"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A2:A5" location="customers!A1" display="customers"/>
+    <hyperlink ref="A6:A9" location="phone!A1" display="phone"/>
+    <hyperlink ref="A10:A13" location="orders!A1" display="orders"/>
+    <hyperlink ref="A18:A21" location="inventory!A1" display="inventory"/>
+    <hyperlink ref="A22:A25" location="coupons!A1" display="coupons"/>
+    <hyperlink ref="A26:A29" location="payments!A1" display="payments"/>
+    <hyperlink ref="A30:A33" location="ware_houses!A1" display="ware_houses"/>
+    <hyperlink ref="A34:A37" location="order_details_inventory!A1" display="order_details_inventory"/>
+    <hyperlink ref="A38:A41" location="customer_coupons!A1" display="customer_coupons"/>
+    <hyperlink ref="A42:A45" location="order_coupons!A1" display="order_coupons"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>
@@ -3274,699 +5832,278 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A2:L162"/>
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" ht="21" spans="1:1">
-      <c r="A2" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="2:2">
-      <c r="B3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="2:2">
-      <c r="B4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="2:2">
-      <c r="B5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2">
-      <c r="B6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2">
-      <c r="B7" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2">
-      <c r="B8" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="9" spans="2:2">
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="10" spans="2:2">
-      <c r="B10" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="13" ht="21" spans="1:1">
-      <c r="A13" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="2:12">
-      <c r="B15" t="s">
-        <v>109</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="16" spans="2:2">
-      <c r="B16" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="2:12">
-      <c r="B17" t="s">
-        <v>112</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2">
-      <c r="B18" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12">
-      <c r="B19" t="s">
-        <v>115</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>116</v>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="14:14">
+      <c r="N6" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" spans="14:14">
+      <c r="N8" s="6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="9" spans="14:18">
+      <c r="N9" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="R9" s="61" t="s">
+        <v>170</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+    <hyperlink ref="R9" location="customer_coupons!A1" display="--&gt; customer_coupons table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="2:2">
-      <c r="B20" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2">
-      <c r="B21" t="s">
-        <v>118</v>
+      <c r="B20" s="5" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="22" spans="2:2">
-      <c r="B22" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="23" spans="2:2">
-      <c r="B23" t="s">
-        <v>107</v>
+      <c r="B22" s="6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="23" customFormat="1" spans="2:6">
+      <c r="B23" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="F23" s="62" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="2:2">
-      <c r="B24" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="26" ht="21" spans="1:1">
-      <c r="A26" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12">
-      <c r="B28" t="s">
-        <v>122</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29" spans="2:2">
-      <c r="B29" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="30" spans="2:12">
-      <c r="B30" t="s">
-        <v>124</v>
-      </c>
-      <c r="L30" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="31" spans="2:2">
-      <c r="B31" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="32" spans="2:12">
-      <c r="B32" t="s">
-        <v>127</v>
-      </c>
-      <c r="L32" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="33" spans="2:2">
-      <c r="B33" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2">
-      <c r="B34" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2">
-      <c r="B35" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2">
-      <c r="B36" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2">
-      <c r="B37" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="40" ht="21" spans="1:1">
-      <c r="A40" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="42" spans="2:12">
-      <c r="B42" t="s">
-        <v>134</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="43" spans="2:2">
-      <c r="B43" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="44" spans="2:12">
-      <c r="B44" t="s">
-        <v>124</v>
-      </c>
-      <c r="L44" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="45" spans="2:2">
-      <c r="B45" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="46" spans="2:2">
-      <c r="B46" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="47" spans="2:2">
-      <c r="B47" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="48" spans="2:2">
-      <c r="B48" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="49" spans="2:2">
-      <c r="B49" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="50" spans="2:2">
-      <c r="B50" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="51" spans="2:2">
-      <c r="B51" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="52" spans="2:2">
-      <c r="B52" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="53" ht="21" spans="1:1">
-      <c r="A53" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="55" spans="2:12">
-      <c r="B55" t="s">
-        <v>144</v>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="56" spans="2:2">
-      <c r="B56" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="57" spans="2:12">
-      <c r="B57" t="s">
-        <v>146</v>
-      </c>
-      <c r="L57" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="58" spans="2:2">
-      <c r="B58" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="59" spans="2:12">
-      <c r="B59" t="s">
-        <v>148</v>
-      </c>
-      <c r="L59" s="3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="60" spans="2:2">
-      <c r="B60" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="61" spans="2:2">
-      <c r="B61" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="62" spans="2:2">
-      <c r="B62" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="63" spans="2:2">
-      <c r="B63" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="64" spans="2:2">
-      <c r="B64" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="65" spans="2:2">
-      <c r="B65" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="69" ht="21" spans="1:1">
-      <c r="A69" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="71" spans="2:2">
-      <c r="B71" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="72" spans="2:2">
-      <c r="B72" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="73" spans="2:2">
-      <c r="B73" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="74" spans="2:2">
-      <c r="B74" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="75" spans="2:2">
-      <c r="B75" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="76" spans="2:2">
-      <c r="B76" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="77" spans="2:2">
-      <c r="B77" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="80" ht="21" spans="1:1">
-      <c r="A80" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="82" spans="2:2">
-      <c r="B82" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="83" spans="2:2">
-      <c r="B83" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="84" spans="2:2">
-      <c r="B84" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="85" spans="2:2">
-      <c r="B85" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="86" spans="2:2">
-      <c r="B86" t="s">
+      <c r="B24" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2">
+      <c r="B25" s="7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+    <hyperlink ref="F23" location="order_coupons!A1" display="--&gt; order_coupons table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="87" spans="2:2">
-      <c r="B87" t="s">
+    <row r="21" spans="3:3">
+      <c r="C21" s="5" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="88" spans="2:2">
-      <c r="B88" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="89" spans="2:2">
-      <c r="B89" t="s">
+    <row r="23" spans="3:3">
+      <c r="C23" s="6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3">
+      <c r="C24" s="7" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="25" spans="3:7">
+      <c r="C25" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="G25" s="61" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3">
+      <c r="C26" s="6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+    <hyperlink ref="G25" location="order_details_inventory!A1" display="--&gt; order_details_inventory table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="14" spans="9:9">
+      <c r="I14" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" spans="9:9">
+      <c r="I16" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="9:13">
+      <c r="I17" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="M17" s="61" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="18" spans="9:9">
+      <c r="I18" s="6" t="s">
+        <v>182</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+    <hyperlink ref="M17" location="order_details_inventory!A1" display="--&gt; order_details_inventory table"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <tabColor theme="4" tint="0.4"/>
+  </sheetPr>
+  <dimension ref="A1:Q7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6"/>
+  <cols>
+    <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="13:13">
+      <c r="M5" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" spans="13:17">
+      <c r="M6" s="7" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="90" spans="2:2">
-      <c r="B90" t="s">
+      <c r="Q6" s="62" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="91" spans="2:2">
-      <c r="B91" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="92" spans="2:2">
-      <c r="B92" t="s">
+    <row r="7" spans="13:17">
+      <c r="M7" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q7" s="62" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="93" spans="2:2">
-      <c r="B93" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="94" spans="2:2">
-      <c r="B94" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="95" spans="2:2">
-      <c r="B95" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="96" spans="2:2">
-      <c r="B96" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="99" ht="21" spans="1:1">
-      <c r="A99" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="101" spans="2:2">
-      <c r="B101" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="102" spans="2:2">
-      <c r="B102" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="103" spans="2:2">
-      <c r="B103" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="104" spans="2:2">
-      <c r="B104" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="105" spans="2:2">
-      <c r="B105" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="106" spans="2:2">
-      <c r="B106" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="107" spans="2:2">
-      <c r="B107" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="108" spans="2:2">
-      <c r="B108" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="109" spans="2:2">
-      <c r="B109" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="112" ht="21" spans="1:1">
-      <c r="A112" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="114" spans="2:2">
-      <c r="B114" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="115" spans="2:2">
-      <c r="B115" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="116" spans="2:2">
-      <c r="B116" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="117" spans="2:2">
-      <c r="B117" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="118" spans="2:2">
-      <c r="B118" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="119" spans="2:2">
-      <c r="B119" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="120" spans="2:2">
-      <c r="B120" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="121" spans="2:2">
-      <c r="B121" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="124" ht="25.8" spans="1:1">
-      <c r="A124" s="4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="126" ht="21" spans="1:1">
-      <c r="A126" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="128" spans="2:2">
-      <c r="B128" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="129" spans="2:2">
-      <c r="B129" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="130" spans="2:2">
-      <c r="B130" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="131" spans="2:2">
-      <c r="B131" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="132" spans="2:2">
-      <c r="B132" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="133" spans="2:2">
-      <c r="B133" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="134" spans="2:2">
-      <c r="B134" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="135" spans="2:2">
-      <c r="B135" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="136" spans="2:2">
-      <c r="B136" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="137" spans="2:2">
-      <c r="B137" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="138" spans="2:2">
-      <c r="B138" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="140" ht="21" spans="1:1">
-      <c r="A140" s="1" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="142" spans="2:2">
-      <c r="B142" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="143" spans="2:2">
-      <c r="B143" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="144" spans="2:2">
-      <c r="B144" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="145" spans="2:2">
-      <c r="B145" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="146" spans="2:2">
-      <c r="B146" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="147" spans="2:2">
-      <c r="B147" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="148" spans="2:2">
-      <c r="B148" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="149" spans="2:2">
-      <c r="B149" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="150" spans="2:2">
-      <c r="B150" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="152" ht="21" spans="1:1">
-      <c r="A152" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="154" spans="2:2">
-      <c r="B154" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="155" spans="2:2">
-      <c r="B155" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="156" spans="2:2">
-      <c r="B156" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="157" spans="2:2">
-      <c r="B157" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="158" spans="2:2">
-      <c r="B158" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="159" spans="2:2">
-      <c r="B159" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="160" spans="2:2">
-      <c r="B160" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="161" spans="2:2">
-      <c r="B161" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="162" spans="2:2">
-      <c r="B162" t="s">
-        <v>202</v>
-      </c>
-    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Table_Interface_summarize!A1" display="Home table"/>
+    <hyperlink ref="Q6" location="customer_coupons!A1" display="--&gt; customer_coupons table"/>
+    <hyperlink ref="Q7" location="order_coupons!A1" display="--&gt; order_coupons table"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
version 36 - Implement Inventory and Warehouse for Detail show product with combined database
</commit_message>
<xml_diff>
--- a/Database_Architecture/Database_design_architecture.xlsx
+++ b/Database_Architecture/Database_design_architecture.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="233">
   <si>
     <t>Model for SQL and No SQL combination</t>
   </si>
@@ -471,6 +471,9 @@
     <t>SQL and NO SQL relationship</t>
   </si>
   <si>
+    <t>Table Index</t>
+  </si>
+  <si>
     <t>Table</t>
   </si>
   <si>
@@ -493,6 +496,9 @@
   </si>
   <si>
     <t>Meaning Ex3</t>
+  </si>
+  <si>
+    <t>Table 1</t>
   </si>
   <si>
     <t>customers</t>
@@ -564,6 +570,9 @@
   </si>
   <si>
     <t>Delete all customer have address "Hanoi", Phone number will be deleted automatically due to config</t>
+  </si>
+  <si>
+    <t>Table 2</t>
   </si>
   <si>
     <t>SELECT phone
@@ -610,6 +619,9 @@
   </si>
   <si>
     <t>Delete all phone number of customer id 4</t>
+  </si>
+  <si>
+    <t>Table 3</t>
   </si>
   <si>
     <t>personal_shopping_bag</t>
@@ -643,6 +655,9 @@
 </t>
   </si>
   <si>
+    <t>Table 4</t>
+  </si>
+  <si>
     <t>orders</t>
   </si>
   <si>
@@ -701,6 +716,9 @@
     <t>Delete all order of customer id 4</t>
   </si>
   <si>
+    <t>Table 5</t>
+  </si>
+  <si>
     <t>order_details</t>
   </si>
   <si>
@@ -742,22 +760,52 @@
     <t>Delete order detail 5</t>
   </si>
   <si>
+    <t>Table 6</t>
+  </si>
+  <si>
     <t>inventory</t>
   </si>
   <si>
+    <t>SELECT quantity FROM inventory WHERE product_sku = '${Product_name}';</t>
+  </si>
+  <si>
+    <t>Read quantity of product based on product name</t>
+  </si>
+  <si>
+    <t>Table 7</t>
+  </si>
+  <si>
     <t>coupons</t>
   </si>
   <si>
+    <t>Table 8</t>
+  </si>
+  <si>
     <t>payments</t>
   </si>
   <si>
+    <t>Table 9</t>
+  </si>
+  <si>
     <t>ware_houses</t>
   </si>
   <si>
+    <t>Table 10</t>
+  </si>
+  <si>
     <t>order_details_inventory</t>
   </si>
   <si>
+    <t>INSERT INTO order_details_inventory (order_detail_id, inventory_id, allocated_quantity) values (3,30,45)</t>
+  </si>
+  <si>
+    <t>Table 11</t>
+  </si>
+  <si>
     <t>customer_coupons</t>
+  </si>
+  <si>
+    <t>Table 12</t>
   </si>
   <si>
     <t>order_coupons</t>
@@ -1630,7 +1678,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -1648,6 +1696,19 @@
       <top style="medium">
         <color auto="1"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
@@ -1712,9 +1773,22 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color auto="1"/>
       </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
@@ -1785,9 +1859,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
+      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
@@ -1843,24 +1915,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
+      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
@@ -2054,7 +2109,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2066,34 +2121,34 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="27" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="27" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2178,7 +2233,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2212,154 +2267,160 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="13" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="17" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -3544,13 +3605,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>243840</xdr:colOff>
       <xdr:row>54</xdr:row>
       <xdr:rowOff>78105</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>914400</xdr:colOff>
       <xdr:row>82</xdr:row>
       <xdr:rowOff>53340</xdr:rowOff>
@@ -3570,7 +3631,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2750820" y="20501610"/>
+          <a:off x="3505200" y="20425410"/>
           <a:ext cx="7581900" cy="5095875"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4493,7 +4554,7 @@
       </c>
     </row>
     <row r="6" spans="4:4">
-      <c r="D6" s="61" t="s">
+      <c r="D6" s="63" t="s">
         <v>3</v>
       </c>
     </row>
@@ -4501,15 +4562,15 @@
       <c r="D7" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="62" t="s">
+      <c r="E7" s="64" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="4:6">
-      <c r="D8" s="63" t="s">
+      <c r="D8" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="63" t="s">
+      <c r="E8" s="65" t="s">
         <v>7</v>
       </c>
       <c r="F8" t="s">
@@ -4517,8 +4578,8 @@
       </c>
     </row>
     <row r="9" spans="4:6">
-      <c r="D9" s="63"/>
-      <c r="E9" s="63"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
       <c r="F9" t="s">
         <v>9</v>
       </c>
@@ -4557,7 +4618,7 @@
       </c>
     </row>
     <row r="17" spans="4:4">
-      <c r="D17" s="61" t="s">
+      <c r="D17" s="63" t="s">
         <v>17</v>
       </c>
     </row>
@@ -4565,7 +4626,7 @@
       <c r="D18" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="62" t="s">
+      <c r="E18" s="64" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4573,7 +4634,7 @@
       <c r="D19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="62" t="s">
+      <c r="E19" s="64" t="s">
         <v>5</v>
       </c>
     </row>
@@ -4593,7 +4654,7 @@
       </c>
     </row>
     <row r="24" spans="4:4">
-      <c r="D24" s="61" t="s">
+      <c r="D24" s="63" t="s">
         <v>23</v>
       </c>
     </row>
@@ -4601,7 +4662,7 @@
       <c r="D25" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="62" t="s">
+      <c r="E25" s="64" t="s">
         <v>24</v>
       </c>
     </row>
@@ -4609,7 +4670,7 @@
       <c r="D26" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="62" t="s">
+      <c r="E26" s="64" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4642,7 +4703,7 @@
       <c r="D33" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="62" t="s">
+      <c r="E33" s="64" t="s">
         <v>30</v>
       </c>
     </row>
@@ -4650,7 +4711,7 @@
       <c r="D34" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="62" t="s">
+      <c r="E34" s="64" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4688,7 +4749,7 @@
       <c r="D42" t="s">
         <v>4</v>
       </c>
-      <c r="E42" s="62" t="s">
+      <c r="E42" s="64" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4701,7 +4762,7 @@
       <c r="D44" t="s">
         <v>19</v>
       </c>
-      <c r="E44" s="62" t="s">
+      <c r="E44" s="64" t="s">
         <v>38</v>
       </c>
     </row>
@@ -4724,7 +4785,7 @@
       <c r="D49" t="s">
         <v>4</v>
       </c>
-      <c r="E49" s="62" t="s">
+      <c r="E49" s="64" t="s">
         <v>38</v>
       </c>
     </row>
@@ -4921,7 +4982,7 @@
       <c r="F66" t="s">
         <v>64</v>
       </c>
-      <c r="G66" s="64" t="s">
+      <c r="G66" s="66" t="s">
         <v>78</v>
       </c>
       <c r="H66" t="s">
@@ -5047,22 +5108,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" spans="16:16">
       <c r="P4" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="16:16">
       <c r="P6" s="7" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="16:16">
       <c r="P7" s="7" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5088,17 +5149,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" spans="9:9">
       <c r="I11" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="9:9">
       <c r="I13" s="6" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -5121,7 +5182,7 @@
   <sheetData>
     <row r="21" spans="1:1">
       <c r="A21" s="1" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -5147,7 +5208,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -5173,7 +5234,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -5199,7 +5260,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -5225,172 +5286,172 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" ht="25.8" spans="2:2">
       <c r="B3" s="2" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" ht="21" spans="2:2">
       <c r="B5" s="3" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="3:3">
       <c r="C8" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" spans="3:3">
       <c r="C9" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="3:3">
       <c r="C10" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" spans="3:3">
       <c r="C11" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="3:3">
       <c r="C12" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="3:3">
       <c r="C13" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="3:3">
       <c r="C14" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
     </row>
     <row r="15" spans="3:3">
       <c r="C15" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="3:3">
       <c r="C16" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" ht="21" spans="2:2">
       <c r="B19" s="3" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="3:3">
       <c r="C22" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
     </row>
     <row r="25" spans="3:3">
       <c r="C25" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
     </row>
     <row r="26" spans="3:3">
       <c r="C26" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
     </row>
     <row r="27" spans="3:3">
       <c r="C27" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
     </row>
     <row r="28" spans="3:3">
       <c r="C28" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
     </row>
     <row r="29" spans="3:3">
       <c r="C29" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" ht="21" spans="2:2">
       <c r="B31" s="3" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
     </row>
     <row r="33" spans="3:3">
       <c r="C33" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" spans="3:3">
       <c r="C34" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35" spans="3:3">
       <c r="C35" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" spans="3:3">
       <c r="C36" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38" spans="3:3">
       <c r="C38" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
     </row>
     <row r="40" spans="3:3">
       <c r="C40" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -5435,20 +5496,21 @@
   <sheetPr>
     <tabColor theme="9" tint="0.4"/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <dimension ref="A1:I49"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25.7777777777778" customWidth="1"/>
-    <col min="2" max="2" width="10.7777777777778" customWidth="1"/>
-    <col min="3" max="3" width="100.777777777778" style="8" customWidth="1"/>
-    <col min="4" max="4" width="40.7777777777778" style="8" customWidth="1"/>
-    <col min="5" max="5" width="80.7777777777778" style="8" customWidth="1"/>
-    <col min="6" max="6" width="40.7777777777778" style="8" customWidth="1"/>
-    <col min="7" max="7" width="80.7777777777778" style="8" customWidth="1"/>
-    <col min="8" max="8" width="40.7777777777778" style="8" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="25.7777777777778" customWidth="1"/>
+    <col min="3" max="3" width="10.7777777777778" customWidth="1"/>
+    <col min="4" max="4" width="100.777777777778" style="8" customWidth="1"/>
+    <col min="5" max="5" width="40.7777777777778" style="8" customWidth="1"/>
+    <col min="6" max="6" width="80.7777777777778" style="8" customWidth="1"/>
+    <col min="7" max="7" width="40.7777777777778" style="8" customWidth="1"/>
+    <col min="8" max="8" width="80.7777777777778" style="8" customWidth="1"/>
+    <col min="9" max="9" width="40.7777777777778" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.15" spans="1:8">
+    <row r="1" ht="15.15" spans="1:9">
       <c r="A1" s="9" t="s">
         <v>99</v>
       </c>
@@ -5470,716 +5532,797 @@
       <c r="G1" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="16" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="2" ht="43.2" spans="1:8">
-      <c r="A2" s="16" t="s">
+      <c r="I1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="17" t="s">
+    </row>
+    <row r="2" ht="43.2" spans="1:9">
+      <c r="A2" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="B2" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="C2" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="D2" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="E2" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="F2" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="H2" s="21"/>
-    </row>
-    <row r="3" ht="57.6" spans="1:8">
-      <c r="A3" s="23"/>
-      <c r="B3" s="24" t="s">
+      <c r="G2" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="H2" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27" t="s">
+      <c r="I2" s="23"/>
+    </row>
+    <row r="3" ht="57.6" spans="1:9">
+      <c r="A3" s="17"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="26" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="D3" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="G3" s="29"/>
-      <c r="H3" s="28"/>
-    </row>
-    <row r="4" ht="57.6" spans="1:8">
-      <c r="A4" s="23"/>
-      <c r="B4" s="24" t="s">
+      <c r="E3" s="28"/>
+      <c r="F3" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="G3" s="30" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="29" t="s">
+      <c r="H3" s="31"/>
+      <c r="I3" s="30"/>
+    </row>
+    <row r="4" ht="57.6" spans="1:9">
+      <c r="A4" s="17"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="H4" s="28"/>
-    </row>
-    <row r="5" ht="43.95" spans="1:8">
-      <c r="A5" s="30"/>
-      <c r="B5" s="31" t="s">
+      <c r="D4" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="E4" s="28"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" ht="43.95" spans="1:9">
+      <c r="A5" s="17"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="D5" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="E5" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="G5" s="36"/>
-      <c r="H5" s="35"/>
-    </row>
-    <row r="6" ht="43.2" spans="1:8">
-      <c r="A6" s="16" t="s">
+      <c r="F5" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="G5" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="H5" s="38"/>
+      <c r="I5" s="37"/>
+    </row>
+    <row r="6" ht="43.2" spans="1:9">
+      <c r="A6" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="B6" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="D6" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="E6" s="38"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="39"/>
-    </row>
-    <row r="7" ht="43.2" spans="1:8">
-      <c r="A7" s="23"/>
-      <c r="B7" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="D7" s="26" t="s">
+      <c r="C6" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="E7" s="27"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="41"/>
-    </row>
-    <row r="8" ht="72" spans="1:8">
-      <c r="A8" s="23"/>
-      <c r="B8" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C8" s="25" t="s">
+      <c r="E6" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="27" t="s">
+      <c r="F6" s="40"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="41"/>
+    </row>
+    <row r="7" ht="43.2" spans="1:9">
+      <c r="A7" s="17"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="E7" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="G8" s="29"/>
-      <c r="H8" s="28"/>
-    </row>
-    <row r="9" ht="43.95" spans="1:8">
-      <c r="A9" s="30"/>
-      <c r="B9" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C9" s="42" t="s">
+      <c r="F7" s="29"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="43"/>
+    </row>
+    <row r="8" ht="72" spans="1:9">
+      <c r="A8" s="17"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="E8" s="28"/>
+      <c r="F8" s="29" t="s">
         <v>134</v>
       </c>
-      <c r="E9" s="44" t="s">
+      <c r="G8" s="30" t="s">
         <v>135</v>
       </c>
-      <c r="F9" s="45" t="s">
+      <c r="H8" s="31"/>
+      <c r="I8" s="30"/>
+    </row>
+    <row r="9" ht="43.95" spans="1:9">
+      <c r="A9" s="17"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="G9" s="46"/>
-      <c r="H9" s="45"/>
-    </row>
-    <row r="10" ht="72" spans="1:8">
-      <c r="A10" s="16" t="s">
+      <c r="E9" s="45" t="s">
         <v>137</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" s="18" t="s">
+      <c r="F9" s="46" t="s">
         <v>138</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="G9" s="47" t="s">
         <v>139</v>
       </c>
-      <c r="E10" s="38"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="39"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="23"/>
-      <c r="B11" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C11" s="25"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="41"/>
-    </row>
-    <row r="12" ht="288" spans="1:8">
-      <c r="A12" s="23"/>
-      <c r="B12" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C12" s="25" t="s">
+      <c r="H9" s="48"/>
+      <c r="I9" s="47"/>
+    </row>
+    <row r="10" ht="72" spans="1:9">
+      <c r="A10" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="D12" s="26"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="28"/>
-    </row>
-    <row r="13" ht="15.15" spans="1:8">
-      <c r="A13" s="30"/>
-      <c r="B13" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="45"/>
-      <c r="G13" s="46"/>
-      <c r="H13" s="45"/>
-    </row>
-    <row r="14" ht="57.6" spans="1:8">
-      <c r="A14" s="16" t="s">
+      <c r="B10" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C14" s="18" t="s">
+      <c r="C10" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D14" s="37" t="s">
+      <c r="E10" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="F10" s="40"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="41"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="17"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D11" s="27"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="43"/>
+    </row>
+    <row r="12" ht="288" spans="1:9">
+      <c r="A12" s="17"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="E12" s="28"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="30"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="17"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D13" s="44"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="47"/>
+      <c r="H13" s="48"/>
+      <c r="I13" s="47"/>
+    </row>
+    <row r="14" ht="57.6" spans="1:9">
+      <c r="A14" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="G14" s="22"/>
-      <c r="H14" s="21"/>
-    </row>
-    <row r="15" ht="43.2" spans="1:8">
-      <c r="A15" s="23"/>
-      <c r="B15" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C15" s="25" t="s">
+      <c r="B14" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="D15" s="47" t="s">
+      <c r="C14" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D14" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="E14" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="F15" s="41" t="s">
+      <c r="F14" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="G15" s="29"/>
-      <c r="H15" s="41"/>
-    </row>
-    <row r="16" ht="43.2" spans="1:8">
-      <c r="A16" s="23"/>
-      <c r="B16" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" s="25" t="s">
+      <c r="G14" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="D16" s="47" t="s">
+      <c r="H14" s="24"/>
+      <c r="I14" s="23"/>
+    </row>
+    <row r="15" ht="43.2" spans="1:9">
+      <c r="A15" s="17"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D15" s="27" t="s">
         <v>151</v>
       </c>
-      <c r="E16" s="48"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="41"/>
-    </row>
-    <row r="17" ht="29.55" spans="1:8">
-      <c r="A17" s="30"/>
-      <c r="B17" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C17" s="42" t="s">
+      <c r="E15" s="49" t="s">
         <v>152</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="F15" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="E17" s="44" t="s">
+      <c r="G15" s="43" t="s">
         <v>154</v>
       </c>
-      <c r="F17" s="45" t="s">
+      <c r="H15" s="31"/>
+      <c r="I15" s="43"/>
+    </row>
+    <row r="16" ht="43.2" spans="1:9">
+      <c r="A16" s="17"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="G17" s="46"/>
-      <c r="H17" s="45"/>
-    </row>
-    <row r="18" ht="43.2" spans="1:8">
-      <c r="A18" s="50" t="s">
+      <c r="E16" s="49" t="s">
         <v>156</v>
       </c>
-      <c r="B18" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C18" s="18" t="s">
+      <c r="F16" s="50"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="51"/>
+      <c r="I16" s="43"/>
+    </row>
+    <row r="17" ht="29.55" spans="1:9">
+      <c r="A17" s="17"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17" s="44" t="s">
         <v>157</v>
       </c>
-      <c r="D18" s="37" t="s">
+      <c r="E17" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="F17" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="G17" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="G18" s="22"/>
-      <c r="H18" s="21"/>
-    </row>
-    <row r="19" ht="43.2" spans="1:8">
-      <c r="A19" s="51"/>
-      <c r="B19" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C19" s="25" t="s">
+      <c r="H17" s="48"/>
+      <c r="I17" s="47"/>
+    </row>
+    <row r="18" ht="43.2" spans="1:9">
+      <c r="A18" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="B18" s="52" t="s">
         <v>162</v>
       </c>
-      <c r="E19" s="48"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="41"/>
-    </row>
-    <row r="20" ht="28.8" spans="1:8">
-      <c r="A20" s="51"/>
-      <c r="B20" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="25" t="s">
+      <c r="C18" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="D20" s="47" t="s">
+      <c r="E18" s="39" t="s">
         <v>164</v>
       </c>
-      <c r="E20" s="48"/>
-      <c r="F20" s="41"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="41"/>
-    </row>
-    <row r="21" ht="29.55" spans="1:8">
-      <c r="A21" s="52"/>
-      <c r="B21" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C21" s="42" t="s">
+      <c r="F18" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="D21" s="43" t="s">
+      <c r="G18" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="E21" s="53"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="45"/>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="16" t="s">
+      <c r="H18" s="24"/>
+      <c r="I18" s="23"/>
+    </row>
+    <row r="19" ht="43.2" spans="1:9">
+      <c r="A19" s="17"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D19" s="27" t="s">
         <v>167</v>
       </c>
-      <c r="B22" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C22" s="55"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="39"/>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="23"/>
-      <c r="B23" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" s="56"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="41"/>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="23"/>
-      <c r="B24" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C24" s="56"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="41"/>
-    </row>
-    <row r="25" ht="15.15" spans="1:8">
-      <c r="A25" s="30"/>
-      <c r="B25" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C25" s="57"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="53"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="45"/>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="16" t="s">
+      <c r="E19" s="28" t="s">
         <v>168</v>
       </c>
-      <c r="B26" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C26" s="55"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="39"/>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="23"/>
-      <c r="B27" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C27" s="56"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="41"/>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" s="23"/>
-      <c r="B28" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C28" s="56"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="41"/>
-      <c r="G28" s="49"/>
-      <c r="H28" s="41"/>
-    </row>
-    <row r="29" ht="15.15" spans="1:8">
-      <c r="A29" s="30"/>
-      <c r="B29" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C29" s="57"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="54"/>
-      <c r="H29" s="45"/>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="16" t="s">
+      <c r="F19" s="50"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="43"/>
+    </row>
+    <row r="20" ht="28.8" spans="1:9">
+      <c r="A20" s="17"/>
+      <c r="B20" s="53"/>
+      <c r="C20" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D20" s="27" t="s">
         <v>169</v>
       </c>
-      <c r="B30" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C30" s="55"/>
-      <c r="D30" s="37"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="39"/>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="23"/>
-      <c r="B31" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C31" s="56"/>
-      <c r="D31" s="47"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="41"/>
-      <c r="G31" s="49"/>
-      <c r="H31" s="41"/>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="23"/>
-      <c r="B32" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C32" s="56"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="49"/>
-      <c r="H32" s="41"/>
-    </row>
-    <row r="33" ht="15.15" spans="1:8">
-      <c r="A33" s="30"/>
-      <c r="B33" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C33" s="57"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="54"/>
-      <c r="H33" s="45"/>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="16" t="s">
+      <c r="E20" s="49" t="s">
         <v>170</v>
       </c>
-      <c r="B34" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="39"/>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="23"/>
-      <c r="B35" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C35" s="56"/>
-      <c r="D35" s="47"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="41"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="41"/>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="23"/>
-      <c r="B36" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C36" s="56"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="41"/>
-      <c r="G36" s="49"/>
-      <c r="H36" s="41"/>
-    </row>
-    <row r="37" ht="15.15" spans="1:8">
-      <c r="A37" s="30"/>
-      <c r="B37" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C37" s="57"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="54"/>
-      <c r="H37" s="45"/>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="58" t="s">
+      <c r="F20" s="50"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="51"/>
+      <c r="I20" s="43"/>
+    </row>
+    <row r="21" ht="29.55" spans="1:9">
+      <c r="A21" s="17"/>
+      <c r="B21" s="54"/>
+      <c r="C21" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D21" s="44" t="s">
         <v>171</v>
       </c>
-      <c r="B38" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="55"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="38"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="40"/>
-      <c r="H38" s="39"/>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="59"/>
-      <c r="B39" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C39" s="56"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="48"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="49"/>
-      <c r="H39" s="41"/>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="59"/>
-      <c r="B40" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C40" s="56"/>
-      <c r="D40" s="47"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="41"/>
-      <c r="G40" s="49"/>
-      <c r="H40" s="41"/>
-    </row>
-    <row r="41" ht="15.15" spans="1:8">
-      <c r="A41" s="60"/>
-      <c r="B41" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C41" s="57"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="53"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="54"/>
-      <c r="H41" s="45"/>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="58" t="s">
+      <c r="E21" s="45" t="s">
         <v>172</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C42" s="55"/>
-      <c r="D42" s="37"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="39"/>
-      <c r="G42" s="40"/>
-      <c r="H42" s="39"/>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="59"/>
-      <c r="B43" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C43" s="56"/>
-      <c r="D43" s="47"/>
-      <c r="E43" s="48"/>
-      <c r="F43" s="41"/>
-      <c r="G43" s="49"/>
-      <c r="H43" s="41"/>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="59"/>
-      <c r="B44" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C44" s="56"/>
-      <c r="D44" s="47"/>
-      <c r="E44" s="48"/>
-      <c r="F44" s="41"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="41"/>
-    </row>
-    <row r="45" ht="15.15" spans="1:8">
-      <c r="A45" s="60"/>
-      <c r="B45" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C45" s="57"/>
-      <c r="D45" s="43"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="45"/>
-      <c r="G45" s="54"/>
-      <c r="H45" s="45"/>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="58" t="s">
+      <c r="F21" s="55"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="56"/>
+      <c r="I21" s="47"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="B46" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C46" s="55"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="39"/>
-      <c r="G46" s="40"/>
-      <c r="H46" s="39"/>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="59"/>
-      <c r="B47" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C47" s="56"/>
-      <c r="D47" s="47"/>
-      <c r="E47" s="48"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="41"/>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" s="59"/>
-      <c r="B48" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C48" s="56"/>
-      <c r="D48" s="47"/>
-      <c r="E48" s="48"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="49"/>
-      <c r="H48" s="41"/>
-    </row>
-    <row r="49" ht="15.15" spans="1:8">
-      <c r="A49" s="60"/>
-      <c r="B49" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C49" s="57"/>
-      <c r="D49" s="43"/>
-      <c r="E49" s="53"/>
-      <c r="F49" s="45"/>
-      <c r="G49" s="54"/>
-      <c r="H49" s="45"/>
+      <c r="B22" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D22" s="57" t="s">
+        <v>175</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>176</v>
+      </c>
+      <c r="F22" s="40"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="41"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="17"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" s="58"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="43"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="17"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" s="58"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="50"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="51"/>
+      <c r="I24" s="43"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="17"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D25" s="59"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="47"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26" s="57"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="41"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="41"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="17"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D27" s="58"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="50"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="43"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="17"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="58"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="50"/>
+      <c r="G28" s="43"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="43"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="17"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D29" s="59"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="47"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="47"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" s="57"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="41"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="17"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="58"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="50"/>
+      <c r="G31" s="43"/>
+      <c r="H31" s="51"/>
+      <c r="I31" s="43"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="17"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D32" s="58"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="50"/>
+      <c r="G32" s="43"/>
+      <c r="H32" s="51"/>
+      <c r="I32" s="43"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="17"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" s="59"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="56"/>
+      <c r="I33" s="47"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D34" s="57"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="41"/>
+      <c r="H34" s="42"/>
+      <c r="I34" s="41"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="17"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D35" s="58"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="50"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="43"/>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="17"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D36" s="58"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="50"/>
+      <c r="G36" s="43"/>
+      <c r="H36" s="51"/>
+      <c r="I36" s="43"/>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="17"/>
+      <c r="B37" s="32"/>
+      <c r="C37" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D37" s="59"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="47"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="47"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="B38" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="C38" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="57"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="40"/>
+      <c r="G38" s="41"/>
+      <c r="H38" s="42"/>
+      <c r="I38" s="41"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="17"/>
+      <c r="B39" s="61"/>
+      <c r="C39" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D39" s="58"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="50"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="51"/>
+      <c r="I39" s="43"/>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="17"/>
+      <c r="B40" s="61"/>
+      <c r="C40" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D40" s="58" t="s">
+        <v>185</v>
+      </c>
+      <c r="E40" s="49"/>
+      <c r="F40" s="50"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="51"/>
+      <c r="I40" s="43"/>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="17"/>
+      <c r="B41" s="62"/>
+      <c r="C41" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D41" s="59"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="47"/>
+      <c r="H41" s="56"/>
+      <c r="I41" s="47"/>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="B42" s="60" t="s">
+        <v>187</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D42" s="57"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="41"/>
+      <c r="H42" s="42"/>
+      <c r="I42" s="41"/>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="17"/>
+      <c r="B43" s="61"/>
+      <c r="C43" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D43" s="58"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="50"/>
+      <c r="G43" s="43"/>
+      <c r="H43" s="51"/>
+      <c r="I43" s="43"/>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="17"/>
+      <c r="B44" s="61"/>
+      <c r="C44" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D44" s="58"/>
+      <c r="E44" s="49"/>
+      <c r="F44" s="50"/>
+      <c r="G44" s="43"/>
+      <c r="H44" s="51"/>
+      <c r="I44" s="43"/>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="17"/>
+      <c r="B45" s="62"/>
+      <c r="C45" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D45" s="59"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="55"/>
+      <c r="G45" s="47"/>
+      <c r="H45" s="56"/>
+      <c r="I45" s="47"/>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="B46" s="60" t="s">
+        <v>189</v>
+      </c>
+      <c r="C46" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D46" s="57"/>
+      <c r="E46" s="39"/>
+      <c r="F46" s="40"/>
+      <c r="G46" s="41"/>
+      <c r="H46" s="42"/>
+      <c r="I46" s="41"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="17"/>
+      <c r="B47" s="61"/>
+      <c r="C47" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D47" s="58"/>
+      <c r="E47" s="49"/>
+      <c r="F47" s="50"/>
+      <c r="G47" s="43"/>
+      <c r="H47" s="51"/>
+      <c r="I47" s="43"/>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="17"/>
+      <c r="B48" s="61"/>
+      <c r="C48" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D48" s="58"/>
+      <c r="E48" s="49"/>
+      <c r="F48" s="50"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="51"/>
+      <c r="I48" s="43"/>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="17"/>
+      <c r="B49" s="62"/>
+      <c r="C49" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D49" s="59"/>
+      <c r="E49" s="45"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="47"/>
+      <c r="H49" s="56"/>
+      <c r="I49" s="47"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="24">
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A10:A13"/>
@@ -6192,19 +6335,31 @@
     <mergeCell ref="A38:A41"/>
     <mergeCell ref="A42:A45"/>
     <mergeCell ref="A46:A49"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="B46:B49"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2:A5" location="customers!A1" display="customers"/>
-    <hyperlink ref="A6:A9" location="phone!A1" display="phone"/>
-    <hyperlink ref="A14:A17" location="orders!A1" display="orders"/>
-    <hyperlink ref="A22:A25" location="inventory!A1" display="inventory"/>
-    <hyperlink ref="A26:A29" location="coupons!A1" display="coupons"/>
-    <hyperlink ref="A30:A33" location="payments!A1" display="payments"/>
-    <hyperlink ref="A34:A37" location="ware_houses!A1" display="ware_houses"/>
-    <hyperlink ref="A38:A41" location="order_details_inventory!A1" display="order_details_inventory"/>
-    <hyperlink ref="A42:A45" location="customer_coupons!A1" display="customer_coupons"/>
-    <hyperlink ref="A46:A49" location="order_coupons!A1" display="order_coupons"/>
-    <hyperlink ref="A10:A13" location="personal_shopping_bag!A1" display="personal_shopping_bag"/>
+    <hyperlink ref="B2:B5" location="customers!A1" display="customers"/>
+    <hyperlink ref="B6:B9" location="phone!A1" display="phone"/>
+    <hyperlink ref="B14:B17" location="orders!A1" display="orders"/>
+    <hyperlink ref="B22:B25" location="inventory!A1" display="inventory"/>
+    <hyperlink ref="B26:B29" location="coupons!A1" display="coupons"/>
+    <hyperlink ref="B30:B33" location="payments!A1" display="payments"/>
+    <hyperlink ref="B34:B37" location="ware_houses!A1" display="ware_houses"/>
+    <hyperlink ref="B38:B41" location="order_details_inventory!A1" display="order_details_inventory"/>
+    <hyperlink ref="B42:B45" location="customer_coupons!A1" display="customer_coupons"/>
+    <hyperlink ref="B46:B49" location="order_coupons!A1" display="order_coupons"/>
+    <hyperlink ref="B10:B13" location="personal_shopping_bag!A1" display="personal_shopping_bag"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -6225,25 +6380,25 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="14:14">
       <c r="N6" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="14:14">
       <c r="N8" s="6" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" spans="14:18">
       <c r="N9" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="R9" s="65" t="s">
-        <v>178</v>
+        <v>193</v>
+      </c>
+      <c r="R9" s="67" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -6270,7 +6425,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -6296,35 +6451,35 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="20" spans="2:2">
       <c r="B20" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="22" spans="2:2">
       <c r="B22" s="6" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
     </row>
     <row r="23" customFormat="1" spans="2:6">
       <c r="B23" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="F23" s="66" t="s">
-        <v>180</v>
+        <v>195</v>
+      </c>
+      <c r="F23" s="68" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="2:2">
       <c r="B24" s="7" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
     </row>
     <row r="25" spans="2:2">
       <c r="B25" s="7" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -6351,35 +6506,35 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" s="6" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" s="7" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" spans="3:7">
       <c r="C25" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="G25" s="65" t="s">
-        <v>186</v>
+        <v>201</v>
+      </c>
+      <c r="G25" s="67" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="26" spans="3:3">
       <c r="C26" s="6" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -6406,30 +6561,30 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="14" spans="9:9">
       <c r="I14" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" spans="9:9">
       <c r="I16" s="6" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" spans="9:13">
       <c r="I17" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="M17" s="65" t="s">
-        <v>186</v>
+        <v>205</v>
+      </c>
+      <c r="M17" s="67" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="18" spans="9:9">
       <c r="I18" s="6" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -6456,28 +6611,28 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="13:13">
       <c r="M5" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="13:17">
       <c r="M6" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="Q6" s="66" t="s">
-        <v>178</v>
+        <v>193</v>
+      </c>
+      <c r="Q6" s="68" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="13:17">
       <c r="M7" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q7" s="66" t="s">
-        <v>180</v>
+        <v>207</v>
+      </c>
+      <c r="Q7" s="68" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>